<commit_message>
Align workbook with Sep 9 import
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R8dce6b1616b44a7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R20f8461391724fc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R63f3503aa61a4806"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R39f6aa95fd3d4945"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="Rb9845a1e90d0469c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R6e8d62f2685446fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R2cd3accae9fc4d5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Rdf917bcb6cf2450f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R2b8d8271aa944d5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R4817fb1a492140e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rd338409f71d74478"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R41f15c41e3524239"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="Ra17a62bfcbe949b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Re84c0c0b40724d21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="Ra37e92f0c0cf43c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R7d34f157624144c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R67dd815b795643e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R113e1022a6f94610"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Rf266c8b308bf481d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="Rc9b85580c6d44334"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R71ed4a4e1be64cdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Rfa48ec52d0be4b5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R395cc778a23e4481"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="Rba81e62b0f414c26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Rdef0ebc893be4770"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R63371b06745143e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R0adc42b3e1364f29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R0b0f34c7f8a64950"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R80f91267578f4cda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="Ra34b38ca413045fe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2776,7 +2776,7 @@
         <x:v>Personal safe cash</x:v>
       </x:c>
       <x:c r="C7" s="42" t="n">
-        <x:v>60</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="D7" s="42" t="n">
         <x:v>0</x:v>
@@ -2785,10 +2785,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="42" t="n">
-        <x:v>60</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="G7" s="36" t="str">
-        <x:v>Wife’s income held as cash; excluded from Wells/Wealthfront funding</x:v>
+        <x:v>Wife’s Sep. 9 income held as cash; excluded from Wells/Wealthfront funding</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -4108,16 +4108,16 @@
         <x:v>Wells Fargo checking</x:v>
       </x:c>
       <x:c r="B4" s="36" t="str">
-        <x:v>Income and recurring payments</x:v>
+        <x:v>Sep. 9 balance + operating history</x:v>
       </x:c>
       <x:c r="C4" s="36" t="str">
-        <x:v>Jul 8-Aug 7, 2026</x:v>
+        <x:v>Sep 9, 2026</x:v>
       </x:c>
       <x:c r="D4" s="36" t="str">
-        <x:v>Weekly $1,343.37 payroll; $75/week automatic Fidelity 401(k) transfer; rent rebuilt at $300 on each of the four Tuesdays after a rent payment; prior $188 weekly Credit Union of Texas car-loan transfers</x:v>
+        <x:v>Available Wells $1,227.78 after pending Fidelity debit; pending payroll $1,343.38; wife’s $160 income is held in the personal safe</x:v>
       </x:c>
       <x:c r="E4" s="36" t="str">
-        <x:v>The prior $805 UMB category was an assumption and has been removed from savings. Rent paid Sep. 1 uses the existing Wealthfront rent bucket; no new rent deposit is made on that payment Tuesday. The next four Tuesday deposits are $300 each ($1,200 total) for the October payment. Fund the car at the annualized rate ($746.47 x 12 / 52) in a reserve, then pay the exact monthly amount on the 27th. An $85 Tuesday Wells Fargo-to-PayPal cruise transfer begins Sep. 1; $50/week is added for a Wealthfront future-expenses fund. AT&amp;T normal baseline is $65/month; Sep. 16 autopay is $88.59 due to a one-time roaming charge.</x:v>
+        <x:v>The earlier Jul–Aug account history establishes the $1,343.37 recurring-payroll baseline and $75 weekly Fidelity transfer. The Sep. 9 balance controls this live review. Rent funding is limited to verified Wells capacity after required actions, not a forced $300 deposit.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -5381,7 +5381,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="5" t="str">
-        <x:v>Use this on payday. Pay or move the listed amounts, then record only unexpected spending below. Statements are a monthly audit, not a required monthly rebuild.</x:v>
+        <x:v>Use this ongoing guide after the live Tuesday Review. It reflects the Sep. 9 import inputs; the current rent contribution is calculated in Tuesday Review and recorded in Savings &amp; Debt.</x:v>
       </x:c>
       <x:c r="B2" s="5"/>
       <x:c r="C2" s="5"/>
@@ -5746,7 +5746,7 @@
       </x:c>
       <x:c r="B25" s="42" t="n">
         <x:f>'Support - Budget Inputs'!D8</x:f>
-        <x:v>1403.37</x:v>
+        <x:v>1503.37</x:v>
       </x:c>
       <x:c r="C25" s="36"/>
       <x:c r="D25" s="36"/>
@@ -5759,7 +5759,7 @@
       </x:c>
       <x:c r="B26" s="217" t="n">
         <x:f>'Support - Budget Inputs'!D7</x:f>
-        <x:v>60</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="C26" s="216"/>
       <x:c r="D26" s="216"/>
@@ -5785,7 +5785,7 @@
       </x:c>
       <x:c r="B28" s="49" t="n">
         <x:f>B25-B23</x:f>
-        <x:v>-128.24466923076943</x:v>
+        <x:v>-28.244669230769432</x:v>
       </x:c>
       <x:c r="C28" s="48"/>
       <x:c r="D28" s="50"/>
@@ -6015,7 +6015,7 @@
       </x:c>
       <x:c r="B6" s="169" t="n">
         <x:f>'Support - Account Snapshots'!F7</x:f>
-        <x:v>60</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="C6" s="178" t="str">
         <x:v>Rent due estimate</x:v>
@@ -6033,7 +6033,7 @@
       </x:c>
       <x:c r="B7" s="180" t="n">
         <x:f>SUM(B5:B6)</x:f>
-        <x:v>11907.64</x:v>
+        <x:v>12007.64</x:v>
       </x:c>
       <x:c r="C7" s="178" t="str">
         <x:v>Tagged rent reserve</x:v>
@@ -6069,7 +6069,7 @@
       </x:c>
       <x:c r="B9" s="170" t="n">
         <x:f>B7-B8</x:f>
-        <x:v>-78.33070000000225</x:v>
+        <x:v>21.669299999997747</x:v>
       </x:c>
       <x:c r="C9" s="183" t="str">
         <x:v>Confirmed funding vs. monthly plan</x:v>
@@ -6587,7 +6587,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="247" t="str">
-        <x:v>History — Closed Weeks</x:v>
+        <x:v>History — Weekly Record</x:v>
       </x:c>
       <x:c r="B1" s="247"/>
       <x:c r="C1" s="247"/>
@@ -6675,7 +6675,7 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="24" customHeight="1">
+    <x:row r="5" ht="42" customHeight="1">
       <x:c r="A5" s="242" t="n">
         <x:v>46266</x:v>
       </x:c>
@@ -6722,7 +6722,7 @@
         <x:v>Legacy baseline: no full line-level source archive existed before the Sep. 9 audit. Do not treat this row as source-certified.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="24" customHeight="1">
+    <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="242" t="n">
         <x:v>46273</x:v>
       </x:c>
@@ -6734,11 +6734,17 @@
         <x:f>A6-1</x:f>
         <x:v>46272</x:v>
       </x:c>
-      <x:c r="D6" s="189"/>
-      <x:c r="E6" s="189"/>
-      <x:c r="F6" s="189"/>
+      <x:c r="D6" s="189" t="n">
+        <x:v>1227.78</x:v>
+      </x:c>
+      <x:c r="E6" s="189" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F6" s="189" t="n">
+        <x:v>1226.78</x:v>
+      </x:c>
       <x:c r="G6" s="188" t="str">
-        <x:v>Data verified — Sep 9</x:v>
+        <x:v>Plan created — Sep 9</x:v>
       </x:c>
       <x:c r="H6" s="189" t="n">
         <x:v>476.6607692307693</x:v>
@@ -6760,7 +6766,7 @@
         <x:v>26.17076923076928</x:v>
       </x:c>
       <x:c r="M6" s="188" t="str">
-        <x:v>Reviewed Wed Sep. 9 because of the holiday delay. Source-controlled import includes the Citi activity correction.</x:v>
+        <x:v>Reviewed Wed Sep. 9 because of the holiday delay. The source-controlled import is verified and the $1,226.78 cash plan is ready for execution; it is not marked completed yet.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
@@ -7591,7 +7597,7 @@
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="G5:G30">
-      <x:formula1>"In progress,Data verified — Sep 9,Legacy — not source-audited,✓ Completed,Needs review"</x:formula1>
+      <x:formula1>"In progress,Plan created — Sep 9,Data verified — Sep 9,Legacy — not source-audited,✓ Completed,Needs review"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14526,17 +14532,17 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="36" t="str">
-        <x:v>Wife income (variable — personal safe)</x:v>
+        <x:v>Wife income (personal safe — Sep 9 actual)</x:v>
       </x:c>
       <x:c r="B7" s="36" t="str">
         <x:v>Weekly</x:v>
       </x:c>
       <x:c r="C7" s="41" t="n">
-        <x:v>60</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="D7" s="42" t="n">
         <x:f>IF(B7="Weekly",C7,C7*12/52)</x:f>
-        <x:v>60</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="E7" s="36"/>
       <x:c r="F7" s="36"/>
@@ -14549,7 +14555,7 @@
       <x:c r="C8" s="43"/>
       <x:c r="D8" s="44" t="n">
         <x:f>SUM(D6:D7)</x:f>
-        <x:v>1403.37</x:v>
+        <x:v>1503.37</x:v>
       </x:c>
       <x:c r="E8" s="36"/>
       <x:c r="F8" s="36"/>
@@ -15046,7 +15052,7 @@
       <x:c r="D34" s="49"/>
       <x:c r="E34" s="49" t="n">
         <x:f>D8-E32</x:f>
-        <x:v>-128.24466923076943</x:v>
+        <x:v>-28.244669230769432</x:v>
       </x:c>
       <x:c r="F34" s="50"/>
     </x:row>

</xml_diff>

<commit_message>
Record additional personal safe income
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R7d34f157624144c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R67dd815b795643e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R113e1022a6f94610"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Rf266c8b308bf481d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="Rc9b85580c6d44334"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R71ed4a4e1be64cdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Rfa48ec52d0be4b5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R395cc778a23e4481"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="Rba81e62b0f414c26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Rdef0ebc893be4770"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R63371b06745143e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R0adc42b3e1364f29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R0b0f34c7f8a64950"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R80f91267578f4cda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="Ra34b38ca413045fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="Rf398eaa1560b4adf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R312c22abc6d6419d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R8bab0e0419bd49f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Rfe035943d3584a4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R0c52b85a53f34508"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R6adddfb3df154af3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R3e4a55aab8b8449d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R94b85015d2ea4cb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R6989b51a9e164106"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R95ff324414fc4c6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R4e5ae8a4bf7d4d9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="Rfddbde0f9c9d4251"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R5effc21d8585403f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Ra7a5f222eafa4b11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R27e6824df9c24744"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2776,7 +2776,7 @@
         <x:v>Personal safe cash</x:v>
       </x:c>
       <x:c r="C7" s="42" t="n">
-        <x:v>160</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="D7" s="42" t="n">
         <x:v>0</x:v>
@@ -2785,10 +2785,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="42" t="n">
-        <x:v>160</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="G7" s="36" t="str">
-        <x:v>Wife’s Sep. 9 income held as cash; excluded from Wells/Wealthfront funding</x:v>
+        <x:v>Wife’s Sep. 9 income held as cash; $160 added to the prior $60. Excluded from Wells/Wealthfront funding.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -4114,7 +4114,7 @@
         <x:v>Sep 9, 2026</x:v>
       </x:c>
       <x:c r="D4" s="36" t="str">
-        <x:v>Available Wells $1,227.78 after pending Fidelity debit; pending payroll $1,343.38; wife’s $160 income is held in the personal safe</x:v>
+        <x:v>Available Wells $1,227.78 after pending Fidelity debit; pending payroll $1,343.38; wife’s $220 total income is held in the personal safe</x:v>
       </x:c>
       <x:c r="E4" s="36" t="str">
         <x:v>The earlier Jul–Aug account history establishes the $1,343.37 recurring-payroll baseline and $75 weekly Fidelity transfer. The Sep. 9 balance controls this live review. Rent funding is limited to verified Wells capacity after required actions, not a forced $300 deposit.</x:v>
@@ -5746,7 +5746,7 @@
       </x:c>
       <x:c r="B25" s="42" t="n">
         <x:f>'Support - Budget Inputs'!D8</x:f>
-        <x:v>1503.37</x:v>
+        <x:v>1563.37</x:v>
       </x:c>
       <x:c r="C25" s="36"/>
       <x:c r="D25" s="36"/>
@@ -5759,7 +5759,7 @@
       </x:c>
       <x:c r="B26" s="217" t="n">
         <x:f>'Support - Budget Inputs'!D7</x:f>
-        <x:v>160</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="C26" s="216"/>
       <x:c r="D26" s="216"/>
@@ -5785,7 +5785,7 @@
       </x:c>
       <x:c r="B28" s="49" t="n">
         <x:f>B25-B23</x:f>
-        <x:v>-28.244669230769432</x:v>
+        <x:v>31.755330769230568</x:v>
       </x:c>
       <x:c r="C28" s="48"/>
       <x:c r="D28" s="50"/>
@@ -6015,7 +6015,7 @@
       </x:c>
       <x:c r="B6" s="169" t="n">
         <x:f>'Support - Account Snapshots'!F7</x:f>
-        <x:v>160</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="C6" s="178" t="str">
         <x:v>Rent due estimate</x:v>
@@ -6033,7 +6033,7 @@
       </x:c>
       <x:c r="B7" s="180" t="n">
         <x:f>SUM(B5:B6)</x:f>
-        <x:v>12007.64</x:v>
+        <x:v>12067.64</x:v>
       </x:c>
       <x:c r="C7" s="178" t="str">
         <x:v>Tagged rent reserve</x:v>
@@ -6069,7 +6069,7 @@
       </x:c>
       <x:c r="B9" s="170" t="n">
         <x:f>B7-B8</x:f>
-        <x:v>21.669299999997747</x:v>
+        <x:v>81.66929999999775</x:v>
       </x:c>
       <x:c r="C9" s="183" t="str">
         <x:v>Confirmed funding vs. monthly plan</x:v>
@@ -14532,17 +14532,17 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="36" t="str">
-        <x:v>Wife income (personal safe — Sep 9 actual)</x:v>
+        <x:v>Wife income (personal safe — Sep 9 total)</x:v>
       </x:c>
       <x:c r="B7" s="36" t="str">
         <x:v>Weekly</x:v>
       </x:c>
       <x:c r="C7" s="41" t="n">
-        <x:v>160</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="D7" s="42" t="n">
         <x:f>IF(B7="Weekly",C7,C7*12/52)</x:f>
-        <x:v>160</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="E7" s="36"/>
       <x:c r="F7" s="36"/>
@@ -14555,7 +14555,7 @@
       <x:c r="C8" s="43"/>
       <x:c r="D8" s="44" t="n">
         <x:f>SUM(D6:D7)</x:f>
-        <x:v>1503.37</x:v>
+        <x:v>1563.37</x:v>
       </x:c>
       <x:c r="E8" s="36"/>
       <x:c r="F8" s="36"/>
@@ -15052,7 +15052,7 @@
       <x:c r="D34" s="49"/>
       <x:c r="E34" s="49" t="n">
         <x:f>D8-E32</x:f>
-        <x:v>-28.244669230769432</x:v>
+        <x:v>31.755330769230568</x:v>
       </x:c>
       <x:c r="F34" s="50"/>
     </x:row>

</xml_diff>

<commit_message>
Regenerate budget workbook from current builder
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="Rf398eaa1560b4adf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R312c22abc6d6419d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R8bab0e0419bd49f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Rfe035943d3584a4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R0c52b85a53f34508"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R6adddfb3df154af3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R3e4a55aab8b8449d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R94b85015d2ea4cb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R6989b51a9e164106"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R95ff324414fc4c6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R4e5ae8a4bf7d4d9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="Rfddbde0f9c9d4251"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R5effc21d8585403f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Ra7a5f222eafa4b11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R27e6824df9c24744"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="Rba18838499cf4a6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Rd93fb7a100674c45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="Rdd9f984027b4483f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Rcbb60a861807497a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R846af412b47e4e74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R46890bf36ef0464e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R1b52cd76d74c4d4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Rff817b8e88004d72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="Rfab73a1dbf9f4da9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Rf45b14a99b8647f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R654ac55aed664095"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R03b507273b2f4a0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R2212354bf1974d39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Rcc24325d07224147"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R8604b36102634008"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Clarify Nationwide pet insurance allocation
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="Rba18838499cf4a6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Rd93fb7a100674c45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="Rdd9f984027b4483f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Rcbb60a861807497a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R846af412b47e4e74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R46890bf36ef0464e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R1b52cd76d74c4d4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Rff817b8e88004d72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="Rfab73a1dbf9f4da9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Rf45b14a99b8647f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R654ac55aed664095"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R03b507273b2f4a0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R2212354bf1974d39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Rcc24325d07224147"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R8604b36102634008"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R6086c57efebf46f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R008fe77a5cd842ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="Rbb229010cea64a3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Rd904b14ef5db496d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="Rfd39959521da4793"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="Rc04da9df1bbe4552"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R83f1f046232b481e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Ra79412a9bbed43f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="Rdf1335c2861a4555"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R6452a32044574189"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R30575320ea054184"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R310f3391558144b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R1dac5b1eb40d4422"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R0835bd802e3a4617"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R2165ea6366c74dc9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5653,7 +5653,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="36" t="str">
-        <x:v>Pet</x:v>
+        <x:v>Pet care + Nationwide insurance</x:v>
       </x:c>
       <x:c r="B19" s="42" t="n">
         <x:f>'Support - Budget Inputs'!E26</x:f>
@@ -5663,7 +5663,7 @@
         <x:v>Use as weekly envelope</x:v>
       </x:c>
       <x:c r="D19" s="36" t="str">
-        <x:v>Formula from weekly budget</x:v>
+        <x:v>Includes $48.27/month Nationwide pet insurance</x:v>
       </x:c>
       <x:c r="E19" s="36"/>
       <x:c r="F19" s="36"/>
@@ -5781,11 +5781,11 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="47" t="str">
-        <x:v>Household weekly buffer / shortfall</x:v>
+        <x:v>Weekly buffer / shortfall from banking income</x:v>
       </x:c>
       <x:c r="B28" s="49" t="n">
-        <x:f>B25-B23</x:f>
-        <x:v>31.755330769230568</x:v>
+        <x:f>B27-B23</x:f>
+        <x:v>-188.24466923076943</x:v>
       </x:c>
       <x:c r="C28" s="48"/>
       <x:c r="D28" s="50"/>
@@ -15387,7 +15387,7 @@
         <x:v>Pet</x:v>
       </x:c>
       <x:c r="B11" s="173" t="str">
-        <x:v>BudgetPetCare + grooming</x:v>
+        <x:v>Nationwide insurance + BudgetPetCare + grooming</x:v>
       </x:c>
       <x:c r="C11" s="248" t="n">
         <x:f>'Support - Budget Inputs'!E26</x:f>

</xml_diff>

<commit_message>
Mark automatic transfers done in Tuesday Review
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="Rd6c0d134c11b4c7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R89b34f3634104d05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R28119a27c9cb479f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R04814f1484da4b05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R02ecf9df589a446c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="Rcba7abf432ba43dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R2395564062f44e72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R9a05857416684f14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R54317c2a17f3427d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R684dfd8a8a0445e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Ra4cbf5fe36ee4e29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="Refd189a4a42a4f58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R081d8886e9044352"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R660cb61b351d474a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R1f6970fb754948dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R8680f6dd342149e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Rbe2ffdc4096a48ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R9dd9cb422ca34209"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Rbe77311ed4a84312"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R555dd8c26dde464e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R64747f67acd8486a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R7f55fcdfd49c484e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Red0e40b1cfc94df0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R5c3cdc40f6104cfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R7696725fa0914ef0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Re01bcc785712437d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R86c32bf2a72f4bfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R8b6efbda20c34993"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Rd47c5298df364203"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R81124eeafab14937"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5242,8 +5242,8 @@
         <x:v>Sep 1–Sep 7 purchases</x:v>
       </x:c>
       <x:c r="C6" s="393" t="str">
-        <x:f>COUNTIF(F9:F19,"✓ Done")&amp;" / "&amp;COUNTA(B9:B19)&amp;" actions completed"</x:f>
-        <x:v>1 / 11 actions completed</x:v>
+        <x:f>COUNTIF(F9:F19,"Done")&amp;" / "&amp;COUNTA(B9:B19)&amp;" actions completed"</x:f>
+        <x:v>4 / 11 actions completed</x:v>
       </x:c>
       <x:c r="D6" s="393" t="str">
         <x:v>Use now</x:v>
@@ -5430,7 +5430,7 @@
       </x:c>
       <x:c r="E15" s="395"/>
       <x:c r="F15" s="404" t="str">
-        <x:v>✓ Done</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G15" s="362" t="str">
         <x:v>Do not count again in cash required</x:v>
@@ -5451,7 +5451,7 @@
       </x:c>
       <x:c r="E16" s="395"/>
       <x:c r="F16" s="404" t="str">
-        <x:v>Scheduled</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G16" s="362" t="str">
         <x:v>Included in cash required; confirm after it posts</x:v>
@@ -5472,7 +5472,7 @@
       </x:c>
       <x:c r="E17" s="395"/>
       <x:c r="F17" s="404" t="str">
-        <x:v>Scheduled</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G17" s="362" t="str">
         <x:v>Included in cash required; confirm after it posts</x:v>
@@ -5493,7 +5493,7 @@
       </x:c>
       <x:c r="E18" s="395"/>
       <x:c r="F18" s="404" t="str">
-        <x:v>Scheduled</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G18" s="362" t="str">
         <x:v>Included in cash required; confirm after it posts</x:v>
@@ -5603,7 +5603,7 @@
   </x:mergeCells>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="F9:F19">
-      <x:formula1>"Not done,✓ Done,Not due,Scheduled,Deferred,Partial"</x:formula1>
+      <x:formula1>"Not done,Done,✓ Done,Not due,Scheduled,Deferred,Partial"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Promote polished workbook as main copy
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R8680f6dd342149e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Rbe2ffdc4096a48ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R9dd9cb422ca34209"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Rbe77311ed4a84312"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R555dd8c26dde464e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R64747f67acd8486a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R7f55fcdfd49c484e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Red0e40b1cfc94df0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R5c3cdc40f6104cfa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R7696725fa0914ef0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Re01bcc785712437d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R86c32bf2a72f4bfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R8b6efbda20c34993"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Rd47c5298df364203"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R81124eeafab14937"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R6f6fde561c3f491f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R1a67045b52a24eb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R9c4c2cf399b94c60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R2d08efb0edda43fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="Rd3ddf2c687514154"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R8566afad8e744fab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R85f4c16fec7b4abc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Re967410d93a1466c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R766f33863c88424e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R7f80bbc84b854878"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R1b6a7984461e4f32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R4b15b3dcf01048ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R544422b8de8d4dbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Raab1e6aa63ab4311"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="Ree1306e0197b4ec5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2570,6 +2570,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF173F5F"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="29" hidden="0" customWidth="1"/>
@@ -2902,6 +2905,9 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFCBD5E1"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
@@ -3207,6 +3213,9 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFCBD5E1"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
@@ -3450,6 +3459,9 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFCBD5E1"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
@@ -3978,6 +3990,9 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFCBD5E1"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
@@ -4440,6 +4455,9 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFCBD5E1"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
@@ -4947,6 +4965,9 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFCBD5E1"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
@@ -5163,6 +5184,9 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF173F5F"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
@@ -5612,6 +5636,9 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF173F5F"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="29" hidden="0" customWidth="1"/>
@@ -6245,6 +6272,9 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF6B4F9B"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
@@ -6829,6 +6859,9 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF0F766E"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
@@ -7454,6 +7487,9 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF566575"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="17" hidden="0" customWidth="1"/>
@@ -8492,6 +8528,9 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFCBD5E1"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
@@ -15350,6 +15389,9 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFCBD5E1"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
@@ -16049,6 +16091,9 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFCBD5E1"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>

</xml_diff>

<commit_message>
Exclude personal safe income from cash plan
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R6f6fde561c3f491f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R1a67045b52a24eb8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R9c4c2cf399b94c60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R2d08efb0edda43fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="Rd3ddf2c687514154"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R8566afad8e744fab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R85f4c16fec7b4abc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Re967410d93a1466c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R766f33863c88424e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="R7f80bbc84b854878"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R1b6a7984461e4f32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R4b15b3dcf01048ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R544422b8de8d4dbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="Raab1e6aa63ab4311"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="Ree1306e0197b4ec5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R05c9632189474eb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Rab5b53a9dfac4b74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="Rcda536e589074692"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R1a4a0b916bca4c83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R370bd46d5f624597"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="Rb81f56e531bd4a2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Rf2d1f9acfab24e8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R7ff3f238ba024ffb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="Rd63df3d526874574"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Rf34858d6597d4605"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rfcd1c5c17b714e3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R13c14963ef374241"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="Rdd751b484e7c4b74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R6879fe08dfab4994"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R8e2fed3642c84911"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -654,14 +654,14 @@
     <x:xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -697,6 +697,9 @@
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
@@ -704,9 +707,6 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5021,10 +5021,10 @@
         <x:v>Sep 9, 2026</x:v>
       </x:c>
       <x:c r="D4" s="362" t="str">
-        <x:v>Available Wells $1,227.78 after pending Fidelity debit; pending payroll $1,343.38; wife’s $220 total income is held in the personal safe</x:v>
+        <x:v>Available Wells $1,227.78 after pending Fidelity debit; personal-safe balance $220 includes the earlier $60 plus an additional $160</x:v>
       </x:c>
       <x:c r="E4" s="362" t="str">
-        <x:v>The earlier Jul–Aug account history establishes the $1,343.37 recurring-payroll baseline and $75 weekly Fidelity transfer. The Sep. 9 balance controls this live review. Rent funding is limited to verified Wells capacity after required actions, not a forced $300 deposit.</x:v>
+        <x:v>The earlier Jul–Aug account history establishes the $1,343.37 recurring-payroll baseline and $75 weekly Fidelity transfer. Personal-safe cash is savings-only and excluded from Wells cash-plan and spending-capacity calculations. The Sep. 9 Wells balance controls this live review.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -6658,11 +6658,11 @@
     </x:row>
     <x:row r="25" ht="25" customHeight="1">
       <x:c r="A25" s="362" t="str">
-        <x:v>Total weekly household income</x:v>
+        <x:v>Usable weekly income — Wells plan</x:v>
       </x:c>
       <x:c r="B25" s="445" t="n">
         <x:f>'Support - Budget Inputs'!D8</x:f>
-        <x:v>1563.37</x:v>
+        <x:v>1343.37</x:v>
       </x:c>
       <x:c r="C25" s="362"/>
       <x:c r="D25" s="362"/>
@@ -6671,10 +6671,10 @@
     </x:row>
     <x:row r="26" ht="25" customHeight="1">
       <x:c r="A26" s="401" t="str">
-        <x:v>Personal-safe income — included in household total</x:v>
+        <x:v>Personal-safe balance — savings only</x:v>
       </x:c>
       <x:c r="B26" s="446" t="n">
-        <x:f>'Support - Budget Inputs'!D7</x:f>
+        <x:f>'Support - Account Snapshots'!F7</x:f>
         <x:v>220</x:v>
       </x:c>
       <x:c r="C26" s="401"/>
@@ -6684,10 +6684,10 @@
     </x:row>
     <x:row r="27" ht="25" customHeight="1">
       <x:c r="A27" s="393" t="str">
-        <x:v>Banking income available for Wells plan</x:v>
+        <x:v>Income used by this plan</x:v>
       </x:c>
       <x:c r="B27" s="447" t="n">
-        <x:f>B25-B26</x:f>
+        <x:f>B25</x:f>
         <x:v>1343.37</x:v>
       </x:c>
       <x:c r="C27" s="393"/>
@@ -6697,7 +6697,7 @@
     </x:row>
     <x:row r="28" ht="25" customHeight="1">
       <x:c r="A28" s="436" t="str">
-        <x:v>Weekly buffer / shortfall from banking income</x:v>
+        <x:v>Weekly buffer / shortfall from Wells income</x:v>
       </x:c>
       <x:c r="B28" s="448" t="n">
         <x:f>B27-B23</x:f>
@@ -15475,30 +15475,30 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="362" t="str">
-        <x:v>Wife income (personal safe — Sep 9 total)</x:v>
+        <x:v>Personal-safe balance (excluded from Wells plan)</x:v>
       </x:c>
       <x:c r="B7" s="362" t="str">
-        <x:v>Weekly</x:v>
-      </x:c>
-      <x:c r="C7" s="396" t="n">
+        <x:v>Balance</x:v>
+      </x:c>
+      <x:c r="C7" s="394" t="n">
+        <x:f>'Support - Account Snapshots'!F7</x:f>
         <x:v>220</x:v>
       </x:c>
-      <x:c r="D7" s="416" t="n">
-        <x:f>IF(B7="Weekly",C7,C7*12/52)</x:f>
-        <x:v>220</x:v>
+      <x:c r="D7" s="394" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E7" s="362"/>
       <x:c r="F7" s="362"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="417" t="str">
-        <x:v>Total net income</x:v>
+        <x:v>Usable weekly income — Wells plan</x:v>
       </x:c>
       <x:c r="B8" s="417"/>
-      <x:c r="C8" s="417"/>
+      <x:c r="C8" s="418"/>
       <x:c r="D8" s="418" t="n">
-        <x:f>SUM(D6:D7)</x:f>
-        <x:v>1563.37</x:v>
+        <x:f>D6</x:f>
+        <x:v>1343.37</x:v>
       </x:c>
       <x:c r="E8" s="362"/>
       <x:c r="F8" s="362"/>
@@ -15995,7 +15995,7 @@
       <x:c r="D34" s="437"/>
       <x:c r="E34" s="437" t="n">
         <x:f>D8-E32</x:f>
-        <x:v>31.755330769230568</x:v>
+        <x:v>-188.24466923076943</x:v>
       </x:c>
       <x:c r="F34" s="439"/>
     </x:row>

</xml_diff>

<commit_message>
Relabel Fidelity transfer as Roth IRA
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R05c9632189474eb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Rab5b53a9dfac4b74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="Rcda536e589074692"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R1a4a0b916bca4c83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R370bd46d5f624597"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="Rb81f56e531bd4a2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="Rf2d1f9acfab24e8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R7ff3f238ba024ffb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="Rd63df3d526874574"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Rf34858d6597d4605"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rfcd1c5c17b714e3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R13c14963ef374241"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="Rdd751b484e7c4b74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R6879fe08dfab4994"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R8e2fed3642c84911"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="Rd99719b0078b4bd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Rd3305aaae7964f0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R699f6b3090244759"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Rb00db621722645b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R71f8582e29304588"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R3e1861bacdef47c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R67d51dfed13c41dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Ra5b9cdefb41d4b49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R43d1c89a6ebb49de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Rcf20d5580f65424e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R67b7455b383d4672"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R0eae1fde02f54517"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="Raf5bcc4c0f2b473d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R680e87be54cc4bd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R4feb8ff3c0fc4f3a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4861,7 +4861,7 @@
         <x:v>Fidelity</x:v>
       </x:c>
       <x:c r="B25" s="581" t="str">
-        <x:v>Fidelity 401(k)</x:v>
+        <x:v>Fidelity Roth IRA</x:v>
       </x:c>
       <x:c r="C25" s="581" t="str">
         <x:v>Transfer / verify</x:v>
@@ -5444,7 +5444,7 @@
         <x:v>Automatic</x:v>
       </x:c>
       <x:c r="B15" s="362" t="str">
-        <x:v>Fidelity 401(k)</x:v>
+        <x:v>Fidelity Roth IRA</x:v>
       </x:c>
       <x:c r="C15" s="362" t="str">
         <x:v>Pending; already in Wells available balance</x:v>
@@ -6603,14 +6603,14 @@
     </x:row>
     <x:row r="21" ht="38" customHeight="1">
       <x:c r="A21" s="362" t="str">
-        <x:v>Fidelity + PayPal savings buckets</x:v>
+        <x:v>Fidelity Roth IRA + PayPal savings buckets</x:v>
       </x:c>
       <x:c r="B21" s="416" t="n">
         <x:f>'Support - Budget Inputs'!E27</x:f>
         <x:v>403.36</x:v>
       </x:c>
       <x:c r="C21" s="362" t="str">
-        <x:v>$75 Fidelity plus $85 cruise, $193.36 tuition, and $50 future fund automatically</x:v>
+        <x:v>$75 Roth IRA plus $85 cruise, $193.36 tuition, and $50 future fund automatically</x:v>
       </x:c>
       <x:c r="D21" s="362" t="str">
         <x:v>Formula from weekly budget</x:v>
@@ -7036,7 +7036,7 @@
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="362" t="str">
-        <x:v>Fidelity 401(k)</x:v>
+        <x:v>Fidelity Roth IRA</x:v>
       </x:c>
       <x:c r="B13" s="395" t="n">
         <x:v>75</x:v>
@@ -15864,7 +15864,7 @@
         <x:v>Savings</x:v>
       </x:c>
       <x:c r="B27" s="362" t="str">
-        <x:v>Fidelity + PayPal savings buckets</x:v>
+        <x:v>Fidelity Roth IRA + PayPal savings buckets</x:v>
       </x:c>
       <x:c r="C27" s="362" t="str">
         <x:v>Weekly</x:v>
@@ -15878,7 +15878,7 @@
         <x:v>403.36</x:v>
       </x:c>
       <x:c r="F27" s="362" t="str">
-        <x:v>$75 Fidelity plus automatic PayPal savings for cruise, tuition, and future expenses</x:v>
+        <x:v>$75 Roth IRA transfer plus automatic PayPal savings for cruise, tuition, and future expenses</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -16641,7 +16641,7 @@
         <x:v>Automatic</x:v>
       </x:c>
       <x:c r="B25" s="362" t="str">
-        <x:v>Fidelity 401(k)</x:v>
+        <x:v>Fidelity Roth IRA</x:v>
       </x:c>
       <x:c r="C25" s="362" t="str">
         <x:v>Weekly automatic transfer</x:v>

</xml_diff>

<commit_message>
Clarify automatic transfer checklist semantics
</commit_message>
<xml_diff>
--- a/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
+++ b/outputs/01a04fdf-3751-72e2-88f1-daf19b8b9d1d/comprehensive_budget.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="Rd99719b0078b4bd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="Rd3305aaae7964f0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R699f6b3090244759"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="Rb00db621722645b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R71f8582e29304588"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R3e1861bacdef47c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R67d51dfed13c41dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="Ra5b9cdefb41d4b49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R43d1c89a6ebb49de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Rcf20d5580f65424e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="R67b7455b383d4672"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R0eae1fde02f54517"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="Raf5bcc4c0f2b473d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R680e87be54cc4bd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R4feb8ff3c0fc4f3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Start" sheetId="1" r:id="R4565538089304063"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Tuesday Review" sheetId="2" r:id="R55002e43eb554e20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. This Week" sheetId="3" r:id="R6df0ed9da5ed42a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Money Plan" sheetId="4" r:id="R7e0dfc1259fa4191"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Savings &amp; Debt" sheetId="5" r:id="R1b2f56d55d9b4c40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. History" sheetId="6" r:id="R2a3fde61469249fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Ledger" sheetId="7" r:id="R8021ef8519484e9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Budget Inputs" sheetId="8" r:id="R202ff23997a24c0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Funding Detail" sheetId="9" r:id="R52e008cf3a8c4337"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Debt Detail" sheetId="10" r:id="Ra529a9e7e1044af5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Promo Detail" sheetId="11" r:id="Rb88f4ea7747944e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Account Snapshots" sheetId="12" r:id="R2dbd043a4c3c4f41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Pending Review" sheetId="13" r:id="R0d7eff0af0e04e57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Rules" sheetId="14" r:id="R888a69301d3a46b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support - Sources" sheetId="15" r:id="R51a69a6aeeee42f5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5211,7 +5211,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="377" t="str">
-        <x:v>Use this live checklist after Start is verified. Planned amounts come from the Sep. 9 account snapshots and funding rules. Done means no further action is needed from you; a bank transaction may still be pending settlement. Scheduled means a transfer is expected but not yet confirmed.</x:v>
+        <x:v>Use this live checklist after Start is verified. Done means no manual action is required. Automatic transfers remain part of the cash plan even when marked Done; bank settlement is verified at the next weekly import.</x:v>
       </x:c>
       <x:c r="B2" s="377"/>
       <x:c r="C2" s="377"/>
@@ -5478,7 +5478,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G16" s="362" t="str">
-        <x:v>Included in cash required; confirm after it posts</x:v>
+        <x:v>Automatic commitment; included in cash required</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="28" customHeight="1">
@@ -5499,7 +5499,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G17" s="362" t="str">
-        <x:v>Included in cash required; confirm after it posts</x:v>
+        <x:v>Automatic commitment; included in cash required</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="28" customHeight="1">
@@ -5520,7 +5520,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G18" s="362" t="str">
-        <x:v>Included in cash required; confirm after it posts</x:v>
+        <x:v>Automatic commitment; included in cash required</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="28" customHeight="1">

</xml_diff>